<commit_message>
Podgląd HTML wyniku + dopasowanie szerokości kolumn opisowych
narzedzia/podglad-html.js renderuje arkusz wynikowy do HTML, odtwarzając
scalenia, obrót tekstu i style ramek zapamiętane przez namiastkę
SpreadsheetApp. Pozwala obejrzeć wygląd bez otwierania arkusza — LibreOffice
w tym środowisku nie ładuje plików xlsx, więc konwersja odpadała.

Kolumny opisowe: grupa 40 px, kategoria 74 px (było 34/34) — przy poprzednich
szerokościach etykiety w rodzaju "I zaj. rozszerzone" zawijały się po jednym
słowie i rozpychały wiersze.

npm run demo generuje teraz .html obok .xlsx i .csv.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MbsaA3GmHHqb25GYdLvx3h
</commit_message>
<xml_diff>
--- a/przyklady/wynik/Wniosek_SLO_Brzozowska_Anna.xlsx
+++ b/przyklady/wynik/Wniosek_SLO_Brzozowska_Anna.xlsx
@@ -722,8 +722,8 @@
   <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4.857142857142857" customWidth="1" min="1" max="1"/>
-    <col width="4.857142857142857" customWidth="1" min="2" max="2"/>
+    <col width="5.714285714285714" customWidth="1" min="1" max="1"/>
+    <col width="10.57142857142857" customWidth="1" min="2" max="2"/>
     <col width="35.71428571428572" customWidth="1" min="3" max="3"/>
     <col width="8.571428571428571" customWidth="1" min="4" max="4"/>
     <col width="8.571428571428571" customWidth="1" min="5" max="5"/>

</xml_diff>